<commit_message>
fix(qa): nhan xet Quy 1 cho ho so hoc sinh - bo so lieu nop bai, giong tich cuc
</commit_message>
<xml_diff>
--- a/docs/qa/10Olinda_Q1_nhan-xet.xlsx
+++ b/docs/qa/10Olinda_Q1_nhan-xet.xlsx
@@ -466,7 +466,7 @@
         <v/>
       </c>
       <c r="E5" t="str">
-        <v>Qua kết quả học tập Quý 1, em Hoàng Anh Hà Chi đã nắm được phần lớn kiến thức trọng tâm và làm bài khá đều tay. Em học tốt nhất ở phần mệnh đề và các phép suy luận, nắm được cách làm các dạng cơ bản. Về ý thức, em nộp bài đầy đủ và đúng hạn, đây là nền tảng tốt để tiến bộ tiếp. Sang Quý 2, em nên dành thêm thời gian cho các dạng bài tổng hợp và chủ động hỏi thầy cô ngay khi gặp bài chưa giải được.</v>
+        <v>Trong Quý 1, em Hoàng Anh Hà Chi có thái độ học tập tích cực và nắm được phần lớn kiến thức trọng tâm của chương trình. Em học tốt phần mệnh đề và các phép suy luận toán học và đã nắm được phương pháp giải các dạng bài cơ bản ở nội dung này. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, nếu duy trì được sự chuyên cần và mạnh dạn trao đổi với thầy cô khi gặp bài khó, em sẽ tiến bộ rõ rệt.</v>
       </c>
       <c r="F5" t="str">
         <v/>
@@ -486,7 +486,7 @@
         <v/>
       </c>
       <c r="E6" t="str">
-        <v>Qua kết quả học tập Quý 1, em Hoàng Tuấn Minh đã có cố gắng nhưng kiến thức còn ở mức trung bình, nhiều dạng bài chưa làm chủ được. So với các phần khác, em đỡ vướng nhất ở phần vectơ và các phép toán vectơ. Về ý thức, em nộp bài đầy đủ và đúng hạn, đây là nền tảng tốt để tiến bộ tiếp. Sang Quý 2, em cần làm lại toàn bộ bài tập đã chữa, ghi chép lại các lỗi sai thường gặp và luyện thêm mỗi tuần để bù phần còn hổng.</v>
+        <v>Trong Quý 1, em Hoàng Tuấn Minh đã có nhiều cố gắng và từng bước làm quen với các dạng toán mới của chương trình. Em tiếp thu tốt nhất ở phần vectơ và các phép toán vectơ, đây là nền tảng thuận lợi để em phát triển thêm. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
       </c>
       <c r="F6" t="str">
         <v/>
@@ -506,7 +506,7 @@
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>Qua kết quả học tập Quý 1, em Hồ Khánh Phương đã nắm được phần lớn kiến thức trọng tâm và làm bài khá đều tay. Em đặc biệt vững phần vectơ và các phép toán vectơ, làm bài chính xác và trình bày rõ ràng. Về ý thức, em nộp bài đầy đủ và đúng hạn, đây là nền tảng tốt để tiến bộ tiếp. Sang Quý 2, em nên dành thêm thời gian cho các dạng bài tổng hợp và chủ động hỏi thầy cô ngay khi gặp bài chưa giải được.</v>
+        <v>Trong Quý 1, em Hồ Khánh Phương có thái độ học tập tích cực và nắm được phần lớn kiến thức trọng tâm của chương trình. Em đặc biệt vững phần vectơ và các phép toán vectơ: các bài làm thể hiện sự chính xác và trình bày rõ ràng, mạch lạc. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, nếu duy trì được sự chuyên cần và mạnh dạn trao đổi với thầy cô khi gặp bài khó, em sẽ tiến bộ rõ rệt.</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -526,7 +526,7 @@
         <v/>
       </c>
       <c r="E8" t="str">
-        <v>Qua kết quả học tập Quý 1, em Nguyễn Công Bảo Khánh đã nắm được phần lớn kiến thức trọng tâm và làm bài khá đều tay. Em học tốt nhất ở phần mệnh đề và các phép suy luận, nắm được cách làm các dạng cơ bản. Về ý thức, em nộp bài tương đối đều nhưng vẫn còn bài bỏ trống, cần khắc phục trong Quý 2. Sang Quý 2, em nên dành thêm thời gian cho các dạng bài tổng hợp và chủ động hỏi thầy cô ngay khi gặp bài chưa giải được.</v>
+        <v>Trong Quý 1, em Nguyễn Công Bảo Khánh có thái độ học tập tích cực và nắm được phần lớn kiến thức trọng tâm của chương trình. Em học tốt phần mệnh đề và các phép suy luận toán học và đã nắm được phương pháp giải các dạng bài cơ bản ở nội dung này. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, nếu duy trì được sự chuyên cần và mạnh dạn trao đổi với thầy cô khi gặp bài khó, em sẽ tiến bộ rõ rệt.</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -546,7 +546,7 @@
         <v/>
       </c>
       <c r="E9" t="str">
-        <v>Qua kết quả học tập Quý 1, em Nguyễn Đỗ Khánh Linh đã nắm được phần lớn kiến thức trọng tâm và làm bài khá đều tay. Em học tốt nhất ở phần mệnh đề và các phép suy luận, nắm được cách làm các dạng cơ bản. Về ý thức, em nộp bài tương đối đều nhưng vẫn còn bài bỏ trống, cần khắc phục trong Quý 2. Sang Quý 2, em nên dành thêm thời gian cho các dạng bài tổng hợp và chủ động hỏi thầy cô ngay khi gặp bài chưa giải được.</v>
+        <v>Trong Quý 1, em Nguyễn Đỗ Khánh Linh có thái độ học tập tích cực và nắm được phần lớn kiến thức trọng tâm của chương trình. Em học tốt phần mệnh đề và các phép suy luận toán học và đã nắm được phương pháp giải các dạng bài cơ bản ở nội dung này. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, nếu duy trì được sự chuyên cần và mạnh dạn trao đổi với thầy cô khi gặp bài khó, em sẽ tiến bộ rõ rệt.</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -566,7 +566,7 @@
         <v/>
       </c>
       <c r="E10" t="str">
-        <v>Qua kết quả học tập Quý 1, em Nguyễn Hoàng Gia Linh đã có cố gắng nhưng kiến thức còn ở mức trung bình, nhiều dạng bài chưa làm chủ được. So với các phần khác, em đỡ vướng nhất ở phần mệnh đề và các phép suy luận. Về ý thức, em nộp bài đầy đủ và đúng hạn, đây là nền tảng tốt để tiến bộ tiếp. Sang Quý 2, em cần làm lại toàn bộ bài tập đã chữa, ghi chép lại các lỗi sai thường gặp và luyện thêm mỗi tuần để bù phần còn hổng.</v>
+        <v>Trong Quý 1, em Nguyễn Hoàng Gia Linh đã có nhiều cố gắng và từng bước làm quen với các dạng toán mới của chương trình. Em tiếp thu tốt nhất ở phần mệnh đề và các phép suy luận toán học, đây là nền tảng thuận lợi để em phát triển thêm. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -586,7 +586,7 @@
         <v/>
       </c>
       <c r="E11" t="str">
-        <v>Qua kết quả học tập Quý 1, em Nguyễn Hoàng Minh Châu còn yếu ở nhiều nội dung quan trọng, kết quả chưa phản ánh đúng khả năng của em. So với các phần khác, em đỡ vướng nhất ở phần mệnh đề và các phép suy luận. Phần hệ thức lượng trong tam giác là chỗ em yếu nhất, sai chủ yếu do chưa nắm chắc phương pháp chứ không phải do bất cẩn. Về ý thức, em nộp bài tương đối đều nhưng vẫn còn bài bỏ trống, cần khắc phục trong Quý 2. Sang Quý 2, thầy cô sẽ cùng em hệ thống lại kiến thức nền; em cần đi học đều, làm đủ bài tập cơ bản và không ngại hỏi khi chưa hiểu bài.</v>
+        <v>Trong Quý 1, em Nguyễn Hoàng Minh Châu đã tham gia học tập và có ý thức tiếp thu bài giảng của thầy cô. Em tiếp thu tốt nhất ở phần mệnh đề và các phép suy luận toán học, đây là nền tảng thuận lợi để em phát triển thêm. Để kết quả được toàn diện hơn, em sẽ được thầy cô đồng hành củng cố thêm phần hệ thức lượng trong tam giác trong thời gian tới. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -606,7 +606,7 @@
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>Qua kết quả học tập Quý 1, em Nguyễn Mai Anh đã có cố gắng nhưng kiến thức còn ở mức trung bình, nhiều dạng bài chưa làm chủ được. So với các phần khác, em đỡ vướng nhất ở phần vectơ và các phép toán vectơ. Về ý thức, em nộp bài tương đối đều nhưng vẫn còn bài bỏ trống, cần khắc phục trong Quý 2. Sang Quý 2, em cần làm lại toàn bộ bài tập đã chữa, ghi chép lại các lỗi sai thường gặp và luyện thêm mỗi tuần để bù phần còn hổng.</v>
+        <v>Trong Quý 1, em Nguyễn Mai Anh đã có nhiều cố gắng và từng bước làm quen với các dạng toán mới của chương trình. Em tiếp thu tốt nhất ở phần vectơ và các phép toán vectơ, đây là nền tảng thuận lợi để em phát triển thêm. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -626,7 +626,7 @@
         <v/>
       </c>
       <c r="E13" t="str">
-        <v>Qua kết quả học tập Quý 1, em Nguyễn Ngọc Diễm còn yếu ở nhiều nội dung quan trọng, kết quả chưa phản ánh đúng khả năng của em. Phần bất phương trình và hệ bất phương trình bậc nhất hai ẩn là chỗ em yếu nhất, sai chủ yếu do chưa nắm chắc phương pháp chứ không phải do bất cẩn. Về ý thức, em nộp bài tương đối đều nhưng vẫn còn bài bỏ trống, cần khắc phục trong Quý 2. Sang Quý 2, thầy cô sẽ cùng em hệ thống lại kiến thức nền; em cần đi học đều, làm đủ bài tập cơ bản và không ngại hỏi khi chưa hiểu bài.</v>
+        <v>Trong Quý 1, em Nguyễn Ngọc Diễm đã tham gia học tập và có ý thức tiếp thu bài giảng của thầy cô. Trong các nội dung của Quý 1, em thể hiện sự cố gắng rõ nhất ở phần giá trị lượng giác của góc từ 0° đến 180°. Để kết quả được toàn diện hơn, em sẽ được thầy cô đồng hành củng cố thêm phần bất phương trình và hệ bất phương trình bậc nhất hai ẩn trong thời gian tới. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -646,7 +646,7 @@
         <v/>
       </c>
       <c r="E14" t="str">
-        <v>Qua kết quả học tập Quý 1, em Nguyễn Nhật Huy đã nắm được phần lớn kiến thức trọng tâm và làm bài khá đều tay. Em học tốt nhất ở phần mệnh đề và các phép suy luận, nắm được cách làm các dạng cơ bản. Về ý thức, em nộp bài đầy đủ và đúng hạn, đây là nền tảng tốt để tiến bộ tiếp. Sang Quý 2, em nên dành thêm thời gian cho các dạng bài tổng hợp và chủ động hỏi thầy cô ngay khi gặp bài chưa giải được.</v>
+        <v>Trong Quý 1, em Nguyễn Nhật Huy có thái độ học tập tích cực và nắm được phần lớn kiến thức trọng tâm của chương trình. Em học tốt phần mệnh đề và các phép suy luận toán học và đã nắm được phương pháp giải các dạng bài cơ bản ở nội dung này. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, nếu duy trì được sự chuyên cần và mạnh dạn trao đổi với thầy cô khi gặp bài khó, em sẽ tiến bộ rõ rệt.</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -666,7 +666,7 @@
         <v/>
       </c>
       <c r="E15" t="str">
-        <v>Qua kết quả học tập Quý 1, em Nguyễn Phước Nam Phong còn yếu ở nhiều nội dung quan trọng, kết quả chưa phản ánh đúng khả năng của em. So với các phần khác, em đỡ vướng nhất ở phần vectơ và các phép toán vectơ. Phần hệ thức lượng trong tam giác là chỗ em yếu nhất, sai chủ yếu do chưa nắm chắc phương pháp chứ không phải do bất cẩn. Về ý thức, em nộp bài tương đối đều nhưng vẫn còn bài bỏ trống, cần khắc phục trong Quý 2. Sang Quý 2, thầy cô sẽ cùng em hệ thống lại kiến thức nền; em cần đi học đều, làm đủ bài tập cơ bản và không ngại hỏi khi chưa hiểu bài.</v>
+        <v>Trong Quý 1, em Nguyễn Phước Nam Phong đã tham gia học tập và có ý thức tiếp thu bài giảng của thầy cô. Em tiếp thu tốt nhất ở phần vectơ và các phép toán vectơ, đây là nền tảng thuận lợi để em phát triển thêm. Để kết quả được toàn diện hơn, em sẽ được thầy cô đồng hành củng cố thêm phần hệ thức lượng trong tam giác trong thời gian tới. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
       </c>
       <c r="F15" t="str">
         <v/>
@@ -686,7 +686,7 @@
         <v/>
       </c>
       <c r="E16" t="str">
-        <v>Qua kết quả học tập Quý 1, em Phạm Minh Châu đã có cố gắng nhưng kiến thức còn ở mức trung bình, nhiều dạng bài chưa làm chủ được. Em học tốt nhất ở phần giá trị lượng giác của góc từ 0° đến 180°, nắm được cách làm các dạng cơ bản. Về ý thức, em nộp bài tương đối đều nhưng vẫn còn bài bỏ trống, cần khắc phục trong Quý 2. Sang Quý 2, em cần làm lại toàn bộ bài tập đã chữa, ghi chép lại các lỗi sai thường gặp và luyện thêm mỗi tuần để bù phần còn hổng.</v>
+        <v>Trong Quý 1, em Phạm Minh Châu đã có nhiều cố gắng và từng bước làm quen với các dạng toán mới của chương trình. Em học tốt phần giá trị lượng giác của góc từ 0° đến 180° và đã nắm được phương pháp giải các dạng bài cơ bản ở nội dung này. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -706,7 +706,7 @@
         <v/>
       </c>
       <c r="E17" t="str">
-        <v>Qua kết quả học tập Quý 1, em Phạm Ngọc Linh Chi còn yếu ở nhiều nội dung quan trọng, kết quả chưa phản ánh đúng khả năng của em. So với các phần khác, em đỡ vướng nhất ở phần vectơ và các phép toán vectơ. Phần bất phương trình và hệ bất phương trình bậc nhất hai ẩn là chỗ em yếu nhất, sai chủ yếu do chưa nắm chắc phương pháp chứ không phải do bất cẩn. Về ý thức, em nộp bài đầy đủ và đúng hạn, đây là nền tảng tốt để tiến bộ tiếp. Sang Quý 2, thầy cô sẽ cùng em hệ thống lại kiến thức nền; em cần đi học đều, làm đủ bài tập cơ bản và không ngại hỏi khi chưa hiểu bài.</v>
+        <v>Trong Quý 1, em Phạm Ngọc Linh Chi đã tham gia học tập và có ý thức tiếp thu bài giảng của thầy cô. Em tiếp thu tốt nhất ở phần vectơ và các phép toán vectơ, đây là nền tảng thuận lợi để em phát triển thêm. Để kết quả được toàn diện hơn, em sẽ được thầy cô đồng hành củng cố thêm phần bất phương trình và hệ bất phương trình bậc nhất hai ẩn trong thời gian tới. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -726,7 +726,7 @@
         <v/>
       </c>
       <c r="E18" t="str">
-        <v>Qua kết quả học tập Quý 1, em Trần Anh Thư đã nắm được phần lớn kiến thức trọng tâm và làm bài khá đều tay. Em học tốt nhất ở phần mệnh đề và các phép suy luận, nắm được cách làm các dạng cơ bản. Về ý thức, em nộp bài đầy đủ và đúng hạn, đây là nền tảng tốt để tiến bộ tiếp. Sang Quý 2, em nên dành thêm thời gian cho các dạng bài tổng hợp và chủ động hỏi thầy cô ngay khi gặp bài chưa giải được.</v>
+        <v>Trong Quý 1, em Trần Anh Thư có thái độ học tập tích cực và nắm được phần lớn kiến thức trọng tâm của chương trình. Em học tốt phần mệnh đề và các phép suy luận toán học và đã nắm được phương pháp giải các dạng bài cơ bản ở nội dung này. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, nếu duy trì được sự chuyên cần và mạnh dạn trao đổi với thầy cô khi gặp bài khó, em sẽ tiến bộ rõ rệt.</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -746,7 +746,7 @@
         <v/>
       </c>
       <c r="E19" t="str">
-        <v>Qua kết quả học tập Quý 1, em Trần Hữu Bảo Nam còn yếu ở nhiều nội dung quan trọng, kết quả chưa phản ánh đúng khả năng của em. So với các phần khác, em đỡ vướng nhất ở phần vectơ và các phép toán vectơ. Phần bất phương trình và hệ bất phương trình bậc nhất hai ẩn là chỗ em yếu nhất, sai chủ yếu do chưa nắm chắc phương pháp chứ không phải do bất cẩn. Về ý thức, em nộp bài tương đối đều nhưng vẫn còn bài bỏ trống, cần khắc phục trong Quý 2. Sang Quý 2, thầy cô sẽ cùng em hệ thống lại kiến thức nền; em cần đi học đều, làm đủ bài tập cơ bản và không ngại hỏi khi chưa hiểu bài.</v>
+        <v>Trong Quý 1, em Trần Hữu Bảo Nam đã tham gia học tập và có ý thức tiếp thu bài giảng của thầy cô. Em tiếp thu tốt nhất ở phần vectơ và các phép toán vectơ, đây là nền tảng thuận lợi để em phát triển thêm. Để kết quả được toàn diện hơn, em sẽ được thầy cô đồng hành củng cố thêm phần bất phương trình và hệ bất phương trình bậc nhất hai ẩn trong thời gian tới. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -766,7 +766,7 @@
         <v/>
       </c>
       <c r="E20" t="str">
-        <v>Qua kết quả học tập Quý 1, em Trần Thùy Anh còn yếu ở nhiều nội dung quan trọng, kết quả chưa phản ánh đúng khả năng của em. Phần vectơ và các phép toán vectơ là chỗ em yếu nhất, sai chủ yếu do chưa nắm chắc phương pháp chứ không phải do bất cẩn. Về ý thức, em còn bỏ nhiều bài tập, đây là nguyên nhân chính khiến kết quả chưa cao. Sang Quý 2, thầy cô sẽ cùng em hệ thống lại kiến thức nền; em cần đi học đều, làm đủ bài tập cơ bản và không ngại hỏi khi chưa hiểu bài.</v>
+        <v>Trong Quý 1, em Trần Thùy Anh đã tham gia học tập và có ý thức tiếp thu bài giảng của thầy cô. Trong các nội dung của Quý 1, em thể hiện sự cố gắng rõ nhất ở phần mệnh đề và các phép suy luận toán học. Để kết quả được toàn diện hơn, em sẽ được thầy cô đồng hành củng cố thêm phần vectơ và các phép toán vectơ trong thời gian tới. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -786,7 +786,7 @@
         <v/>
       </c>
       <c r="E21" t="str">
-        <v>Qua kết quả học tập Quý 1, em Trịnh Bảo Nam đã có cố gắng nhưng kiến thức còn ở mức trung bình, nhiều dạng bài chưa làm chủ được. Em học tốt nhất ở phần vectơ và các phép toán vectơ, nắm được cách làm các dạng cơ bản. Về ý thức, em nộp bài tương đối đều nhưng vẫn còn bài bỏ trống, cần khắc phục trong Quý 2. Sang Quý 2, em cần làm lại toàn bộ bài tập đã chữa, ghi chép lại các lỗi sai thường gặp và luyện thêm mỗi tuần để bù phần còn hổng.</v>
+        <v>Trong Quý 1, em Trịnh Bảo Nam đã có nhiều cố gắng và từng bước làm quen với các dạng toán mới của chương trình. Em học tốt phần vectơ và các phép toán vectơ và đã nắm được phương pháp giải các dạng bài cơ bản ở nội dung này. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
       </c>
       <c r="F21" t="str">
         <v/>
@@ -806,7 +806,7 @@
         <v/>
       </c>
       <c r="E22" t="str">
-        <v>Qua kết quả học tập Quý 1, em Vũ Bảo An còn yếu ở nhiều nội dung quan trọng, kết quả chưa phản ánh đúng khả năng của em. Phần vectơ và các phép toán vectơ là chỗ em yếu nhất, sai chủ yếu do chưa nắm chắc phương pháp chứ không phải do bất cẩn. Về ý thức, em nộp bài tương đối đều nhưng vẫn còn bài bỏ trống, cần khắc phục trong Quý 2. Sang Quý 2, thầy cô sẽ cùng em hệ thống lại kiến thức nền; em cần đi học đều, làm đủ bài tập cơ bản và không ngại hỏi khi chưa hiểu bài.</v>
+        <v>Trong Quý 1, em Vũ Bảo An đã tham gia học tập và có ý thức tiếp thu bài giảng của thầy cô. Trong các nội dung của Quý 1, em thể hiện sự cố gắng rõ nhất ở phần mệnh đề và các phép suy luận toán học. Để kết quả được toàn diện hơn, em sẽ được thầy cô đồng hành củng cố thêm phần vectơ và các phép toán vectơ trong thời gian tới. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
       </c>
       <c r="F22" t="str">
         <v/>
@@ -826,7 +826,7 @@
         <v/>
       </c>
       <c r="E23" t="str">
-        <v>Qua kết quả học tập Quý 1, em Vũ Nhật Anh còn yếu ở nhiều nội dung quan trọng, kết quả chưa phản ánh đúng khả năng của em. Phần hệ thức lượng trong tam giác là chỗ em yếu nhất, sai chủ yếu do chưa nắm chắc phương pháp chứ không phải do bất cẩn. Về ý thức, em còn bỏ nhiều bài tập, đây là nguyên nhân chính khiến kết quả chưa cao. Sang Quý 2, thầy cô sẽ cùng em hệ thống lại kiến thức nền; em cần đi học đều, làm đủ bài tập cơ bản và không ngại hỏi khi chưa hiểu bài.</v>
+        <v>Trong Quý 1, em Vũ Nhật Anh đã tham gia học tập và có ý thức tiếp thu bài giảng của thầy cô. Trong các nội dung của Quý 1, em thể hiện sự cố gắng rõ nhất ở phần vectơ và các phép toán vectơ. Để kết quả được toàn diện hơn, em sẽ được thầy cô đồng hành củng cố thêm phần hệ thức lượng trong tam giác trong thời gian tới. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
       </c>
       <c r="F23" t="str">
         <v/>

</xml_diff>

<commit_message>
fix(qa): nhan xet Quy 1 van phong hoc ba, bo dinh huong Quy 2
</commit_message>
<xml_diff>
--- a/docs/qa/10Olinda_Q1_nhan-xet.xlsx
+++ b/docs/qa/10Olinda_Q1_nhan-xet.xlsx
@@ -466,7 +466,7 @@
         <v/>
       </c>
       <c r="E5" t="str">
-        <v>Trong Quý 1, em Hoàng Anh Hà Chi có thái độ học tập tích cực và nắm được phần lớn kiến thức trọng tâm của chương trình. Em học tốt phần mệnh đề và các phép suy luận toán học và đã nắm được phương pháp giải các dạng bài cơ bản ở nội dung này. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, nếu duy trì được sự chuyên cần và mạnh dạn trao đổi với thầy cô khi gặp bài khó, em sẽ tiến bộ rõ rệt.</v>
+        <v>Trong Quý 1, em Hoàng Anh Hà Chi có kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em nắm tốt nội dung mệnh đề và các phép suy luận toán học và thực hiện được các dạng bài cơ bản của phần này. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
       </c>
       <c r="F5" t="str">
         <v/>
@@ -486,7 +486,7 @@
         <v/>
       </c>
       <c r="E6" t="str">
-        <v>Trong Quý 1, em Hoàng Tuấn Minh đã có nhiều cố gắng và từng bước làm quen với các dạng toán mới của chương trình. Em tiếp thu tốt nhất ở phần vectơ và các phép toán vectơ, đây là nền tảng thuận lợi để em phát triển thêm. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
+        <v>Trong Quý 1, em Hoàng Tuấn Minh có kết quả học tập môn Toán ở mức trung bình, đã tiếp thu được các nội dung cơ bản của chương trình. Trong các nội dung của quý, em tiếp thu tốt nhất phần vectơ và các phép toán vectơ. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
       </c>
       <c r="F6" t="str">
         <v/>
@@ -506,7 +506,7 @@
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>Trong Quý 1, em Hồ Khánh Phương có thái độ học tập tích cực và nắm được phần lớn kiến thức trọng tâm của chương trình. Em đặc biệt vững phần vectơ và các phép toán vectơ: các bài làm thể hiện sự chính xác và trình bày rõ ràng, mạch lạc. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, nếu duy trì được sự chuyên cần và mạnh dạn trao đổi với thầy cô khi gặp bài khó, em sẽ tiến bộ rõ rệt.</v>
+        <v>Trong Quý 1, em Hồ Khánh Phương có kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em nắm vững và vận dụng tốt nhất nội dung vectơ và các phép toán vectơ, bài làm thể hiện sự chính xác và trình bày rõ ràng. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -526,7 +526,7 @@
         <v/>
       </c>
       <c r="E8" t="str">
-        <v>Trong Quý 1, em Nguyễn Công Bảo Khánh có thái độ học tập tích cực và nắm được phần lớn kiến thức trọng tâm của chương trình. Em học tốt phần mệnh đề và các phép suy luận toán học và đã nắm được phương pháp giải các dạng bài cơ bản ở nội dung này. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, nếu duy trì được sự chuyên cần và mạnh dạn trao đổi với thầy cô khi gặp bài khó, em sẽ tiến bộ rõ rệt.</v>
+        <v>Trong Quý 1, em Nguyễn Công Bảo Khánh có kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em nắm tốt nội dung mệnh đề và các phép suy luận toán học và thực hiện được các dạng bài cơ bản của phần này. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -546,7 +546,7 @@
         <v/>
       </c>
       <c r="E9" t="str">
-        <v>Trong Quý 1, em Nguyễn Đỗ Khánh Linh có thái độ học tập tích cực và nắm được phần lớn kiến thức trọng tâm của chương trình. Em học tốt phần mệnh đề và các phép suy luận toán học và đã nắm được phương pháp giải các dạng bài cơ bản ở nội dung này. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, nếu duy trì được sự chuyên cần và mạnh dạn trao đổi với thầy cô khi gặp bài khó, em sẽ tiến bộ rõ rệt.</v>
+        <v>Trong Quý 1, em Nguyễn Đỗ Khánh Linh có kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em nắm tốt nội dung mệnh đề và các phép suy luận toán học và thực hiện được các dạng bài cơ bản của phần này. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -566,7 +566,7 @@
         <v/>
       </c>
       <c r="E10" t="str">
-        <v>Trong Quý 1, em Nguyễn Hoàng Gia Linh đã có nhiều cố gắng và từng bước làm quen với các dạng toán mới của chương trình. Em tiếp thu tốt nhất ở phần mệnh đề và các phép suy luận toán học, đây là nền tảng thuận lợi để em phát triển thêm. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
+        <v>Trong Quý 1, em Nguyễn Hoàng Gia Linh có kết quả học tập môn Toán ở mức trung bình, đã tiếp thu được các nội dung cơ bản của chương trình. Trong các nội dung của quý, em tiếp thu tốt nhất phần mệnh đề và các phép suy luận toán học. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -586,7 +586,7 @@
         <v/>
       </c>
       <c r="E11" t="str">
-        <v>Trong Quý 1, em Nguyễn Hoàng Minh Châu đã tham gia học tập và có ý thức tiếp thu bài giảng của thầy cô. Em tiếp thu tốt nhất ở phần mệnh đề và các phép suy luận toán học, đây là nền tảng thuận lợi để em phát triển thêm. Để kết quả được toàn diện hơn, em sẽ được thầy cô đồng hành củng cố thêm phần hệ thức lượng trong tam giác trong thời gian tới. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
+        <v>Trong Quý 1, em Nguyễn Hoàng Minh Châu đã tham gia học tập và bước đầu tiếp cận các nội dung của chương trình Toán. Trong các nội dung của quý, em tiếp thu tốt nhất phần mệnh đề và các phép suy luận toán học. Nội dung hệ thức lượng trong tam giác cần được củng cố thêm để kết quả học tập của em được đồng đều hơn.</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -606,7 +606,7 @@
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>Trong Quý 1, em Nguyễn Mai Anh đã có nhiều cố gắng và từng bước làm quen với các dạng toán mới của chương trình. Em tiếp thu tốt nhất ở phần vectơ và các phép toán vectơ, đây là nền tảng thuận lợi để em phát triển thêm. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
+        <v>Trong Quý 1, em Nguyễn Mai Anh có kết quả học tập môn Toán ở mức trung bình, đã tiếp thu được các nội dung cơ bản của chương trình. Trong các nội dung của quý, em tiếp thu tốt nhất phần vectơ và các phép toán vectơ. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -626,7 +626,7 @@
         <v/>
       </c>
       <c r="E13" t="str">
-        <v>Trong Quý 1, em Nguyễn Ngọc Diễm đã tham gia học tập và có ý thức tiếp thu bài giảng của thầy cô. Trong các nội dung của Quý 1, em thể hiện sự cố gắng rõ nhất ở phần giá trị lượng giác của góc từ 0° đến 180°. Để kết quả được toàn diện hơn, em sẽ được thầy cô đồng hành củng cố thêm phần bất phương trình và hệ bất phương trình bậc nhất hai ẩn trong thời gian tới. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
+        <v>Trong Quý 1, em Nguyễn Ngọc Diễm đã tham gia học tập và bước đầu tiếp cận các nội dung của chương trình Toán. Em đạt kết quả cao nhất ở nội dung giá trị lượng giác của góc từ 0° đến 180°. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố thêm để kết quả học tập của em được đồng đều hơn.</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -646,7 +646,7 @@
         <v/>
       </c>
       <c r="E14" t="str">
-        <v>Trong Quý 1, em Nguyễn Nhật Huy có thái độ học tập tích cực và nắm được phần lớn kiến thức trọng tâm của chương trình. Em học tốt phần mệnh đề và các phép suy luận toán học và đã nắm được phương pháp giải các dạng bài cơ bản ở nội dung này. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, nếu duy trì được sự chuyên cần và mạnh dạn trao đổi với thầy cô khi gặp bài khó, em sẽ tiến bộ rõ rệt.</v>
+        <v>Trong Quý 1, em Nguyễn Nhật Huy có kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em nắm tốt nội dung mệnh đề và các phép suy luận toán học và thực hiện được các dạng bài cơ bản của phần này. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -666,7 +666,7 @@
         <v/>
       </c>
       <c r="E15" t="str">
-        <v>Trong Quý 1, em Nguyễn Phước Nam Phong đã tham gia học tập và có ý thức tiếp thu bài giảng của thầy cô. Em tiếp thu tốt nhất ở phần vectơ và các phép toán vectơ, đây là nền tảng thuận lợi để em phát triển thêm. Để kết quả được toàn diện hơn, em sẽ được thầy cô đồng hành củng cố thêm phần hệ thức lượng trong tam giác trong thời gian tới. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
+        <v>Trong Quý 1, em Nguyễn Phước Nam Phong đã tham gia học tập và bước đầu tiếp cận các nội dung của chương trình Toán. Trong các nội dung của quý, em tiếp thu tốt nhất phần vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố thêm để kết quả học tập của em được đồng đều hơn.</v>
       </c>
       <c r="F15" t="str">
         <v/>
@@ -686,7 +686,7 @@
         <v/>
       </c>
       <c r="E16" t="str">
-        <v>Trong Quý 1, em Phạm Minh Châu đã có nhiều cố gắng và từng bước làm quen với các dạng toán mới của chương trình. Em học tốt phần giá trị lượng giác của góc từ 0° đến 180° và đã nắm được phương pháp giải các dạng bài cơ bản ở nội dung này. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
+        <v>Trong Quý 1, em Phạm Minh Châu có kết quả học tập môn Toán ở mức trung bình, đã tiếp thu được các nội dung cơ bản của chương trình. Em nắm tốt nội dung giá trị lượng giác của góc từ 0° đến 180° và thực hiện được các dạng bài cơ bản của phần này. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -706,7 +706,7 @@
         <v/>
       </c>
       <c r="E17" t="str">
-        <v>Trong Quý 1, em Phạm Ngọc Linh Chi đã tham gia học tập và có ý thức tiếp thu bài giảng của thầy cô. Em tiếp thu tốt nhất ở phần vectơ và các phép toán vectơ, đây là nền tảng thuận lợi để em phát triển thêm. Để kết quả được toàn diện hơn, em sẽ được thầy cô đồng hành củng cố thêm phần bất phương trình và hệ bất phương trình bậc nhất hai ẩn trong thời gian tới. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
+        <v>Trong Quý 1, em Phạm Ngọc Linh Chi đã tham gia học tập và bước đầu tiếp cận các nội dung của chương trình Toán. Trong các nội dung của quý, em tiếp thu tốt nhất phần vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố thêm để kết quả học tập của em được đồng đều hơn.</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -726,7 +726,7 @@
         <v/>
       </c>
       <c r="E18" t="str">
-        <v>Trong Quý 1, em Trần Anh Thư có thái độ học tập tích cực và nắm được phần lớn kiến thức trọng tâm của chương trình. Em học tốt phần mệnh đề và các phép suy luận toán học và đã nắm được phương pháp giải các dạng bài cơ bản ở nội dung này. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, nếu duy trì được sự chuyên cần và mạnh dạn trao đổi với thầy cô khi gặp bài khó, em sẽ tiến bộ rõ rệt.</v>
+        <v>Trong Quý 1, em Trần Anh Thư có kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em nắm tốt nội dung mệnh đề và các phép suy luận toán học và thực hiện được các dạng bài cơ bản của phần này. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -746,7 +746,7 @@
         <v/>
       </c>
       <c r="E19" t="str">
-        <v>Trong Quý 1, em Trần Hữu Bảo Nam đã tham gia học tập và có ý thức tiếp thu bài giảng của thầy cô. Em tiếp thu tốt nhất ở phần vectơ và các phép toán vectơ, đây là nền tảng thuận lợi để em phát triển thêm. Để kết quả được toàn diện hơn, em sẽ được thầy cô đồng hành củng cố thêm phần bất phương trình và hệ bất phương trình bậc nhất hai ẩn trong thời gian tới. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
+        <v>Trong Quý 1, em Trần Hữu Bảo Nam đã tham gia học tập và bước đầu tiếp cận các nội dung của chương trình Toán. Trong các nội dung của quý, em tiếp thu tốt nhất phần vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố thêm để kết quả học tập của em được đồng đều hơn.</v>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -766,7 +766,7 @@
         <v/>
       </c>
       <c r="E20" t="str">
-        <v>Trong Quý 1, em Trần Thùy Anh đã tham gia học tập và có ý thức tiếp thu bài giảng của thầy cô. Trong các nội dung của Quý 1, em thể hiện sự cố gắng rõ nhất ở phần mệnh đề và các phép suy luận toán học. Để kết quả được toàn diện hơn, em sẽ được thầy cô đồng hành củng cố thêm phần vectơ và các phép toán vectơ trong thời gian tới. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
+        <v>Trong Quý 1, em Trần Thùy Anh đã tham gia học tập và bước đầu tiếp cận các nội dung của chương trình Toán. Em đạt kết quả cao nhất ở nội dung mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố thêm để kết quả học tập của em được đồng đều hơn.</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -786,7 +786,7 @@
         <v/>
       </c>
       <c r="E21" t="str">
-        <v>Trong Quý 1, em Trịnh Bảo Nam đã có nhiều cố gắng và từng bước làm quen với các dạng toán mới của chương trình. Em học tốt phần vectơ và các phép toán vectơ và đã nắm được phương pháp giải các dạng bài cơ bản ở nội dung này. Các nội dung trong quý đều được em tiếp thu tương đối đồng đều, tạo thuận lợi cho việc học tiếp ở Quý 2. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
+        <v>Trong Quý 1, em Trịnh Bảo Nam có kết quả học tập môn Toán ở mức trung bình, đã tiếp thu được các nội dung cơ bản của chương trình. Em nắm tốt nội dung vectơ và các phép toán vectơ và thực hiện được các dạng bài cơ bản của phần này. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
       </c>
       <c r="F21" t="str">
         <v/>
@@ -806,7 +806,7 @@
         <v/>
       </c>
       <c r="E22" t="str">
-        <v>Trong Quý 1, em Vũ Bảo An đã tham gia học tập và có ý thức tiếp thu bài giảng của thầy cô. Trong các nội dung của Quý 1, em thể hiện sự cố gắng rõ nhất ở phần mệnh đề và các phép suy luận toán học. Để kết quả được toàn diện hơn, em sẽ được thầy cô đồng hành củng cố thêm phần vectơ và các phép toán vectơ trong thời gian tới. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
+        <v>Trong Quý 1, em Vũ Bảo An đã tham gia học tập và bước đầu tiếp cận các nội dung của chương trình Toán. Em đạt kết quả cao nhất ở nội dung mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố thêm để kết quả học tập của em được đồng đều hơn.</v>
       </c>
       <c r="F22" t="str">
         <v/>
@@ -826,7 +826,7 @@
         <v/>
       </c>
       <c r="E23" t="str">
-        <v>Trong Quý 1, em Vũ Nhật Anh đã tham gia học tập và có ý thức tiếp thu bài giảng của thầy cô. Trong các nội dung của Quý 1, em thể hiện sự cố gắng rõ nhất ở phần vectơ và các phép toán vectơ. Để kết quả được toàn diện hơn, em sẽ được thầy cô đồng hành củng cố thêm phần hệ thức lượng trong tam giác trong thời gian tới. Bước sang Quý 2, thầy cô tin rằng với sự đồng hành của gia đình và nhà trường, em sẽ từng bước vững vàng hơn và đạt kết quả tốt hơn.</v>
+        <v>Trong Quý 1, em Vũ Nhật Anh đã tham gia học tập và bước đầu tiếp cận các nội dung của chương trình Toán. Em đạt kết quả cao nhất ở nội dung vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố thêm để kết quả học tập của em được đồng đều hơn.</v>
       </c>
       <c r="F23" t="str">
         <v/>

</xml_diff>

<commit_message>
fix(qa): nhan xet Q1 bo cau so sanh, sua lap tu, bo sung gioi tinh 54 HS
</commit_message>
<xml_diff>
--- a/docs/qa/10Olinda_Q1_nhan-xet.xlsx
+++ b/docs/qa/10Olinda_Q1_nhan-xet.xlsx
@@ -460,13 +460,13 @@
         <v>Hoàng Anh Hà Chi</v>
       </c>
       <c r="C5" t="str">
-        <v/>
+        <v>Nữ</v>
       </c>
       <c r="D5" t="str">
         <v/>
       </c>
       <c r="E5" t="str">
-        <v>Trong Quý 1, em Hoàng Anh Hà Chi có kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em nắm tốt nội dung mệnh đề và các phép suy luận toán học và thực hiện được các dạng bài cơ bản của phần này. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
+        <v>Trong Quý 1, em Hoàng Anh Hà Chi đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học. Các nội dung trong chương trình được em tiếp thu đều.</v>
       </c>
       <c r="F5" t="str">
         <v/>
@@ -480,13 +480,13 @@
         <v>Hoàng Tuấn Minh</v>
       </c>
       <c r="C6" t="str">
-        <v/>
+        <v>Nam</v>
       </c>
       <c r="D6" t="str">
         <v/>
       </c>
       <c r="E6" t="str">
-        <v>Trong Quý 1, em Hoàng Tuấn Minh có kết quả học tập môn Toán ở mức trung bình, đã tiếp thu được các nội dung cơ bản của chương trình. Trong các nội dung của quý, em tiếp thu tốt nhất phần vectơ và các phép toán vectơ. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
+        <v>Trong Quý 1, em Hoàng Tuấn Minh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Các nội dung trong chương trình được em tiếp thu đều.</v>
       </c>
       <c r="F6" t="str">
         <v/>
@@ -500,13 +500,13 @@
         <v>Hồ Khánh Phương</v>
       </c>
       <c r="C7" t="str">
-        <v/>
+        <v>Nữ</v>
       </c>
       <c r="D7" t="str">
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>Trong Quý 1, em Hồ Khánh Phương có kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em nắm vững và vận dụng tốt nhất nội dung vectơ và các phép toán vectơ, bài làm thể hiện sự chính xác và trình bày rõ ràng. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
+        <v>Trong Quý 1, em Hồ Khánh Phương đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em vận dụng tốt nhất vectơ và các phép toán vectơ, bài làm thể hiện sự chính xác và trình bày rõ ràng. Các nội dung trong chương trình được em tiếp thu đều.</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -520,13 +520,13 @@
         <v>Nguyễn Công Bảo Khánh</v>
       </c>
       <c r="C8" t="str">
-        <v/>
+        <v>Nữ</v>
       </c>
       <c r="D8" t="str">
         <v/>
       </c>
       <c r="E8" t="str">
-        <v>Trong Quý 1, em Nguyễn Công Bảo Khánh có kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em nắm tốt nội dung mệnh đề và các phép suy luận toán học và thực hiện được các dạng bài cơ bản của phần này. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
+        <v>Trong Quý 1, em Nguyễn Công Bảo Khánh đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học. Các nội dung trong chương trình được em tiếp thu đều.</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -540,13 +540,13 @@
         <v>Nguyễn Đỗ Khánh Linh</v>
       </c>
       <c r="C9" t="str">
-        <v/>
+        <v>Nữ</v>
       </c>
       <c r="D9" t="str">
         <v/>
       </c>
       <c r="E9" t="str">
-        <v>Trong Quý 1, em Nguyễn Đỗ Khánh Linh có kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em nắm tốt nội dung mệnh đề và các phép suy luận toán học và thực hiện được các dạng bài cơ bản của phần này. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
+        <v>Trong Quý 1, em Nguyễn Đỗ Khánh Linh đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học. Các nội dung trong chương trình được em tiếp thu đều.</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -560,13 +560,13 @@
         <v>Nguyễn Hoàng Gia Linh</v>
       </c>
       <c r="C10" t="str">
-        <v/>
+        <v>Nữ</v>
       </c>
       <c r="D10" t="str">
         <v/>
       </c>
       <c r="E10" t="str">
-        <v>Trong Quý 1, em Nguyễn Hoàng Gia Linh có kết quả học tập môn Toán ở mức trung bình, đã tiếp thu được các nội dung cơ bản của chương trình. Trong các nội dung của quý, em tiếp thu tốt nhất phần mệnh đề và các phép suy luận toán học. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
+        <v>Trong Quý 1, em Nguyễn Hoàng Gia Linh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học. Các nội dung trong chương trình được em tiếp thu đều.</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -580,13 +580,13 @@
         <v>Nguyễn Hoàng Minh Châu</v>
       </c>
       <c r="C11" t="str">
-        <v/>
+        <v>Nữ</v>
       </c>
       <c r="D11" t="str">
         <v/>
       </c>
       <c r="E11" t="str">
-        <v>Trong Quý 1, em Nguyễn Hoàng Minh Châu đã tham gia học tập và bước đầu tiếp cận các nội dung của chương trình Toán. Trong các nội dung của quý, em tiếp thu tốt nhất phần mệnh đề và các phép suy luận toán học. Nội dung hệ thức lượng trong tam giác cần được củng cố thêm để kết quả học tập của em được đồng đều hơn.</v>
+        <v>Trong Quý 1, em Nguyễn Hoàng Minh Châu đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -600,13 +600,13 @@
         <v>Nguyễn Mai Anh</v>
       </c>
       <c r="C12" t="str">
-        <v/>
+        <v>Nữ</v>
       </c>
       <c r="D12" t="str">
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>Trong Quý 1, em Nguyễn Mai Anh có kết quả học tập môn Toán ở mức trung bình, đã tiếp thu được các nội dung cơ bản của chương trình. Trong các nội dung của quý, em tiếp thu tốt nhất phần vectơ và các phép toán vectơ. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
+        <v>Trong Quý 1, em Nguyễn Mai Anh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Các nội dung trong chương trình được em tiếp thu đều.</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -620,13 +620,13 @@
         <v>Nguyễn Ngọc Diễm</v>
       </c>
       <c r="C13" t="str">
-        <v/>
+        <v>Nữ</v>
       </c>
       <c r="D13" t="str">
         <v/>
       </c>
       <c r="E13" t="str">
-        <v>Trong Quý 1, em Nguyễn Ngọc Diễm đã tham gia học tập và bước đầu tiếp cận các nội dung của chương trình Toán. Em đạt kết quả cao nhất ở nội dung giá trị lượng giác của góc từ 0° đến 180°. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố thêm để kết quả học tập của em được đồng đều hơn.</v>
+        <v>Trong Quý 1, em Nguyễn Ngọc Diễm đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em đạt kết quả cao nhất ở giá trị lượng giác của góc từ 0° đến 180°. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -640,13 +640,13 @@
         <v>Nguyễn Nhật Huy</v>
       </c>
       <c r="C14" t="str">
-        <v/>
+        <v>Nam</v>
       </c>
       <c r="D14" t="str">
         <v/>
       </c>
       <c r="E14" t="str">
-        <v>Trong Quý 1, em Nguyễn Nhật Huy có kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em nắm tốt nội dung mệnh đề và các phép suy luận toán học và thực hiện được các dạng bài cơ bản của phần này. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
+        <v>Trong Quý 1, em Nguyễn Nhật Huy đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học. Các nội dung trong chương trình được em tiếp thu đều.</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -660,13 +660,13 @@
         <v>Nguyễn Phước Nam Phong</v>
       </c>
       <c r="C15" t="str">
-        <v/>
+        <v>Nam</v>
       </c>
       <c r="D15" t="str">
         <v/>
       </c>
       <c r="E15" t="str">
-        <v>Trong Quý 1, em Nguyễn Phước Nam Phong đã tham gia học tập và bước đầu tiếp cận các nội dung của chương trình Toán. Trong các nội dung của quý, em tiếp thu tốt nhất phần vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố thêm để kết quả học tập của em được đồng đều hơn.</v>
+        <v>Trong Quý 1, em Nguyễn Phước Nam Phong đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F15" t="str">
         <v/>
@@ -680,13 +680,13 @@
         <v>Phạm Minh Châu</v>
       </c>
       <c r="C16" t="str">
-        <v/>
+        <v>Nữ</v>
       </c>
       <c r="D16" t="str">
         <v/>
       </c>
       <c r="E16" t="str">
-        <v>Trong Quý 1, em Phạm Minh Châu có kết quả học tập môn Toán ở mức trung bình, đã tiếp thu được các nội dung cơ bản của chương trình. Em nắm tốt nội dung giá trị lượng giác của góc từ 0° đến 180° và thực hiện được các dạng bài cơ bản của phần này. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
+        <v>Trong Quý 1, em Phạm Minh Châu đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Em thực hiện tốt các dạng bài của giá trị lượng giác của góc từ 0° đến 180°. Các nội dung trong chương trình được em tiếp thu đều.</v>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -700,13 +700,13 @@
         <v>Phạm Ngọc Linh Chi</v>
       </c>
       <c r="C17" t="str">
-        <v/>
+        <v>Nữ</v>
       </c>
       <c r="D17" t="str">
         <v/>
       </c>
       <c r="E17" t="str">
-        <v>Trong Quý 1, em Phạm Ngọc Linh Chi đã tham gia học tập và bước đầu tiếp cận các nội dung của chương trình Toán. Trong các nội dung của quý, em tiếp thu tốt nhất phần vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố thêm để kết quả học tập của em được đồng đều hơn.</v>
+        <v>Trong Quý 1, em Phạm Ngọc Linh Chi đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -720,13 +720,13 @@
         <v>Trần Anh Thư</v>
       </c>
       <c r="C18" t="str">
-        <v/>
+        <v>Nữ</v>
       </c>
       <c r="D18" t="str">
         <v/>
       </c>
       <c r="E18" t="str">
-        <v>Trong Quý 1, em Trần Anh Thư có kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em nắm tốt nội dung mệnh đề và các phép suy luận toán học và thực hiện được các dạng bài cơ bản của phần này. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
+        <v>Trong Quý 1, em Trần Anh Thư đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học. Các nội dung trong chương trình được em tiếp thu đều.</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -740,13 +740,13 @@
         <v>Trần Hữu Bảo Nam</v>
       </c>
       <c r="C19" t="str">
-        <v/>
+        <v>Nam</v>
       </c>
       <c r="D19" t="str">
         <v/>
       </c>
       <c r="E19" t="str">
-        <v>Trong Quý 1, em Trần Hữu Bảo Nam đã tham gia học tập và bước đầu tiếp cận các nội dung của chương trình Toán. Trong các nội dung của quý, em tiếp thu tốt nhất phần vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố thêm để kết quả học tập của em được đồng đều hơn.</v>
+        <v>Trong Quý 1, em Trần Hữu Bảo Nam đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -760,13 +760,13 @@
         <v>Trần Thùy Anh</v>
       </c>
       <c r="C20" t="str">
-        <v/>
+        <v>Nữ</v>
       </c>
       <c r="D20" t="str">
         <v/>
       </c>
       <c r="E20" t="str">
-        <v>Trong Quý 1, em Trần Thùy Anh đã tham gia học tập và bước đầu tiếp cận các nội dung của chương trình Toán. Em đạt kết quả cao nhất ở nội dung mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố thêm để kết quả học tập của em được đồng đều hơn.</v>
+        <v>Trong Quý 1, em Trần Thùy Anh đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -780,13 +780,13 @@
         <v>Trịnh Bảo Nam</v>
       </c>
       <c r="C21" t="str">
-        <v/>
+        <v>Nam</v>
       </c>
       <c r="D21" t="str">
         <v/>
       </c>
       <c r="E21" t="str">
-        <v>Trong Quý 1, em Trịnh Bảo Nam có kết quả học tập môn Toán ở mức trung bình, đã tiếp thu được các nội dung cơ bản của chương trình. Em nắm tốt nội dung vectơ và các phép toán vectơ và thực hiện được các dạng bài cơ bản của phần này. Các nội dung trong quý được em tiếp thu tương đối đồng đều.</v>
+        <v>Trong Quý 1, em Trịnh Bảo Nam đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Em thực hiện tốt các dạng bài của vectơ và các phép toán vectơ. Các nội dung trong chương trình được em tiếp thu đều.</v>
       </c>
       <c r="F21" t="str">
         <v/>
@@ -800,13 +800,13 @@
         <v>Vũ Bảo An</v>
       </c>
       <c r="C22" t="str">
-        <v/>
+        <v>Nam</v>
       </c>
       <c r="D22" t="str">
         <v/>
       </c>
       <c r="E22" t="str">
-        <v>Trong Quý 1, em Vũ Bảo An đã tham gia học tập và bước đầu tiếp cận các nội dung của chương trình Toán. Em đạt kết quả cao nhất ở nội dung mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố thêm để kết quả học tập của em được đồng đều hơn.</v>
+        <v>Trong Quý 1, em Vũ Bảo An đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F22" t="str">
         <v/>
@@ -820,13 +820,13 @@
         <v>Vũ Nhật Anh</v>
       </c>
       <c r="C23" t="str">
-        <v/>
+        <v>Nam</v>
       </c>
       <c r="D23" t="str">
         <v/>
       </c>
       <c r="E23" t="str">
-        <v>Trong Quý 1, em Vũ Nhật Anh đã tham gia học tập và bước đầu tiếp cận các nội dung của chương trình Toán. Em đạt kết quả cao nhất ở nội dung vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố thêm để kết quả học tập của em được đồng đều hơn.</v>
+        <v>Trong Quý 1, em Vũ Nhật Anh đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em đạt kết quả cao nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F23" t="str">
         <v/>

</xml_diff>

<commit_message>
feat(qa): nhan xet Q1 phan hoa theo hanh vi hoc tap tung em
</commit_message>
<xml_diff>
--- a/docs/qa/10Olinda_Q1_nhan-xet.xlsx
+++ b/docs/qa/10Olinda_Q1_nhan-xet.xlsx
@@ -466,7 +466,7 @@
         <v/>
       </c>
       <c r="E5" t="str">
-        <v>Trong Quý 1, em Hoàng Anh Hà Chi đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học. Các nội dung trong chương trình được em tiếp thu đều.</v>
+        <v>Trong Quý 1, em Hoàng Anh Hà Chi đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Điểm nổi bật là em làm tốt hơn hẳn khi kiểm tra tập trung so với luyện tập thường ngày, cho thấy em có khả năng huy động kiến thức dưới áp lực thời gian. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F5" t="str">
         <v/>
@@ -486,7 +486,7 @@
         <v/>
       </c>
       <c r="E6" t="str">
-        <v>Trong Quý 1, em Hoàng Tuấn Minh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Các nội dung trong chương trình được em tiếp thu đều.</v>
+        <v>Trong Quý 1, em Hoàng Tuấn Minh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Điểm đáng ghi nhận là em có tiến bộ rõ rệt về sau: kết quả những bài cuối quý cao hơn hẳn giai đoạn đầu, cho thấy em đã điều chỉnh được cách học. Em có kết quả khá nhất ở vectơ và các phép toán vectơ.</v>
       </c>
       <c r="F6" t="str">
         <v/>
@@ -506,7 +506,7 @@
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>Trong Quý 1, em Hồ Khánh Phương đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em vận dụng tốt nhất vectơ và các phép toán vectơ, bài làm thể hiện sự chính xác và trình bày rõ ràng. Các nội dung trong chương trình được em tiếp thu đều.</v>
+        <v>Trong Quý 1, em Hồ Khánh Phương đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Kết quả của em tương đối đồng đều qua các lần kiểm tra, không có giai đoạn nào sa sút rõ rệt. Em nắm vững và vận dụng tốt nhất vectơ và các phép toán vectơ, bài làm thể hiện sự chính xác và trình bày rõ ràng.</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -526,7 +526,7 @@
         <v/>
       </c>
       <c r="E8" t="str">
-        <v>Trong Quý 1, em Nguyễn Công Bảo Khánh đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học. Các nội dung trong chương trình được em tiếp thu đều.</v>
+        <v>Trong Quý 1, em Nguyễn Công Bảo Khánh đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Điểm đáng ghi nhận là em có tiến bộ rõ rệt về sau: kết quả những bài cuối quý cao hơn hẳn giai đoạn đầu, cho thấy em đã điều chỉnh được cách học. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -546,7 +546,7 @@
         <v/>
       </c>
       <c r="E9" t="str">
-        <v>Trong Quý 1, em Nguyễn Đỗ Khánh Linh đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học. Các nội dung trong chương trình được em tiếp thu đều.</v>
+        <v>Trong Quý 1, em Nguyễn Đỗ Khánh Linh đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm. Kết quả các bài cuối quý có phần giảm so với giai đoạn đầu, rất có thể do khối lượng kiến thức tăng nhanh ở giai đoạn ôn thi giữa kì. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -566,7 +566,7 @@
         <v/>
       </c>
       <c r="E10" t="str">
-        <v>Trong Quý 1, em Nguyễn Hoàng Gia Linh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học. Các nội dung trong chương trình được em tiếp thu đều.</v>
+        <v>Trong Quý 1, em Nguyễn Hoàng Gia Linh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Kết quả của em tương đối đồng đều qua các lần kiểm tra, không có giai đoạn nào sa sút rõ rệt. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -586,7 +586,7 @@
         <v/>
       </c>
       <c r="E11" t="str">
-        <v>Trong Quý 1, em Nguyễn Hoàng Minh Châu đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Nguyễn Hoàng Minh Châu đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Kết quả của em tương đối đồng đều qua các lần kiểm tra, không có giai đoạn nào sa sút rõ rệt. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -606,7 +606,7 @@
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>Trong Quý 1, em Nguyễn Mai Anh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Các nội dung trong chương trình được em tiếp thu đều.</v>
+        <v>Trong Quý 1, em Nguyễn Mai Anh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Kết quả giữa các lần kiểm tra của em có độ chênh khá lớn: có lần làm rất tốt nhưng cũng có lần còn ở mức thấp, cho thấy phong độ chưa thật ổn định. Em có kết quả khá nhất ở vectơ và các phép toán vectơ.</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -626,7 +626,7 @@
         <v/>
       </c>
       <c r="E13" t="str">
-        <v>Trong Quý 1, em Nguyễn Ngọc Diễm đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em đạt kết quả cao nhất ở giá trị lượng giác của góc từ 0° đến 180°. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Nguyễn Ngọc Diễm đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Kết quả các bài cuối quý có phần giảm so với giai đoạn đầu, rất có thể do khối lượng kiến thức tăng nhanh ở giai đoạn ôn thi giữa kì. Em đạt kết quả cao nhất ở giá trị lượng giác của góc từ 0° đến 180°. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -646,7 +646,7 @@
         <v/>
       </c>
       <c r="E14" t="str">
-        <v>Trong Quý 1, em Nguyễn Nhật Huy đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học. Các nội dung trong chương trình được em tiếp thu đều.</v>
+        <v>Trong Quý 1, em Nguyễn Nhật Huy đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Điểm nổi bật là em làm tốt hơn hẳn khi kiểm tra tập trung so với luyện tập thường ngày, cho thấy em có khả năng huy động kiến thức dưới áp lực thời gian. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -666,7 +666,7 @@
         <v/>
       </c>
       <c r="E15" t="str">
-        <v>Trong Quý 1, em Nguyễn Phước Nam Phong đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Nguyễn Phước Nam Phong đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Kết quả các bài cuối quý có phần giảm so với giai đoạn đầu, rất có thể do khối lượng kiến thức tăng nhanh ở giai đoạn ôn thi giữa kì. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F15" t="str">
         <v/>
@@ -686,7 +686,7 @@
         <v/>
       </c>
       <c r="E16" t="str">
-        <v>Trong Quý 1, em Phạm Minh Châu đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Em thực hiện tốt các dạng bài của giá trị lượng giác của góc từ 0° đến 180°. Các nội dung trong chương trình được em tiếp thu đều.</v>
+        <v>Trong Quý 1, em Phạm Minh Châu đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Kết quả các bài cuối quý có phần giảm so với giai đoạn đầu, rất có thể do khối lượng kiến thức tăng nhanh ở giai đoạn ôn thi giữa kì. Em thực hiện tốt các dạng bài của giá trị lượng giác của góc từ 0° đến 180°.</v>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -706,7 +706,7 @@
         <v/>
       </c>
       <c r="E17" t="str">
-        <v>Trong Quý 1, em Phạm Ngọc Linh Chi đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Phạm Ngọc Linh Chi đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Điểm đáng ghi nhận là em có tiến bộ rõ rệt về sau: kết quả những bài cuối quý cao hơn hẳn giai đoạn đầu, cho thấy em đã điều chỉnh được cách học. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -726,7 +726,7 @@
         <v/>
       </c>
       <c r="E18" t="str">
-        <v>Trong Quý 1, em Trần Anh Thư đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm của chương trình. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học. Các nội dung trong chương trình được em tiếp thu đều.</v>
+        <v>Trong Quý 1, em Trần Anh Thư đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Điểm đáng ghi nhận là em có tiến bộ rõ rệt về sau: kết quả những bài cuối quý cao hơn hẳn giai đoạn đầu, cho thấy em đã điều chỉnh được cách học. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -746,7 +746,7 @@
         <v/>
       </c>
       <c r="E19" t="str">
-        <v>Trong Quý 1, em Trần Hữu Bảo Nam đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Trần Hữu Bảo Nam đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Kết quả của em tương đối đồng đều qua các lần kiểm tra, không có giai đoạn nào sa sút rõ rệt. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -766,7 +766,7 @@
         <v/>
       </c>
       <c r="E20" t="str">
-        <v>Trong Quý 1, em Trần Thùy Anh đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Trần Thùy Anh đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Kết quả các bài cuối quý có phần giảm so với giai đoạn đầu, rất có thể do khối lượng kiến thức tăng nhanh ở giai đoạn ôn thi giữa kì. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -786,7 +786,7 @@
         <v/>
       </c>
       <c r="E21" t="str">
-        <v>Trong Quý 1, em Trịnh Bảo Nam đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Em thực hiện tốt các dạng bài của vectơ và các phép toán vectơ. Các nội dung trong chương trình được em tiếp thu đều.</v>
+        <v>Trong Quý 1, em Trịnh Bảo Nam đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Kết quả của em tương đối đồng đều qua các lần kiểm tra, không có giai đoạn nào sa sút rõ rệt. Em thực hiện tốt các dạng bài của vectơ và các phép toán vectơ.</v>
       </c>
       <c r="F21" t="str">
         <v/>
@@ -806,7 +806,7 @@
         <v/>
       </c>
       <c r="E22" t="str">
-        <v>Trong Quý 1, em Vũ Bảo An đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Vũ Bảo An đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Kết quả các bài cuối quý có phần giảm so với giai đoạn đầu, rất có thể do khối lượng kiến thức tăng nhanh ở giai đoạn ôn thi giữa kì. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F22" t="str">
         <v/>
@@ -826,7 +826,7 @@
         <v/>
       </c>
       <c r="E23" t="str">
-        <v>Trong Quý 1, em Vũ Nhật Anh đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em đạt kết quả cao nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Vũ Nhật Anh đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Điểm nổi bật là em làm tốt hơn hẳn khi kiểm tra tập trung so với luyện tập thường ngày, cho thấy em có khả năng huy động kiến thức dưới áp lực thời gian. Em đạt kết quả cao nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F23" t="str">
         <v/>

</xml_diff>

<commit_message>
feat(qa): nhan xet Q1 dua tren kieu loi tung cau cua moi em
</commit_message>
<xml_diff>
--- a/docs/qa/10Olinda_Q1_nhan-xet.xlsx
+++ b/docs/qa/10Olinda_Q1_nhan-xet.xlsx
@@ -466,7 +466,7 @@
         <v/>
       </c>
       <c r="E5" t="str">
-        <v>Trong Quý 1, em Hoàng Anh Hà Chi đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Điểm nổi bật là em làm tốt hơn hẳn khi kiểm tra tập trung so với luyện tập thường ngày, cho thấy em có khả năng huy động kiến thức dưới áp lực thời gian. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Hoàng Anh Hà Chi đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Điều cần lưu ý là các bài tự luận của em còn thiếu bước lập luận hoặc thiếu kết luận, dù hướng làm đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F5" t="str">
         <v/>
@@ -486,7 +486,7 @@
         <v/>
       </c>
       <c r="E6" t="str">
-        <v>Trong Quý 1, em Hoàng Tuấn Minh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Điểm đáng ghi nhận là em có tiến bộ rõ rệt về sau: kết quả những bài cuối quý cao hơn hẳn giai đoạn đầu, cho thấy em đã điều chỉnh được cách học. Em có kết quả khá nhất ở vectơ và các phép toán vectơ.</v>
+        <v>Trong Quý 1, em Hoàng Tuấn Minh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Khi làm bài, em còn để trống một số câu, phần lớn rơi vào các câu khó hoặc câu cuối đề. Em có kết quả khá nhất ở vectơ và các phép toán vectơ.</v>
       </c>
       <c r="F6" t="str">
         <v/>
@@ -506,7 +506,7 @@
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>Trong Quý 1, em Hồ Khánh Phương đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Kết quả của em tương đối đồng đều qua các lần kiểm tra, không có giai đoạn nào sa sút rõ rệt. Em nắm vững và vận dụng tốt nhất vectơ và các phép toán vectơ, bài làm thể hiện sự chính xác và trình bày rõ ràng.</v>
+        <v>Trong Quý 1, em Hồ Khánh Phương đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Đáng chú ý là phần lớn câu hỏi em đều làm đúng, số câu sai không nhiều và thường chỉ là lỗi nhỏ. Em nắm vững và vận dụng tốt nhất vectơ và các phép toán vectơ, bài làm thể hiện sự chính xác và trình bày rõ ràng.</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -526,7 +526,7 @@
         <v/>
       </c>
       <c r="E8" t="str">
-        <v>Trong Quý 1, em Nguyễn Công Bảo Khánh đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Điểm đáng ghi nhận là em có tiến bộ rõ rệt về sau: kết quả những bài cuối quý cao hơn hẳn giai đoạn đầu, cho thấy em đã điều chỉnh được cách học. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Nguyễn Công Bảo Khánh đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Điều cần lưu ý là các bài tự luận của em còn thiếu bước lập luận hoặc thiếu kết luận, dù hướng làm đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -546,7 +546,7 @@
         <v/>
       </c>
       <c r="E9" t="str">
-        <v>Trong Quý 1, em Nguyễn Đỗ Khánh Linh đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm. Kết quả các bài cuối quý có phần giảm so với giai đoạn đầu, rất có thể do khối lượng kiến thức tăng nhanh ở giai đoạn ôn thi giữa kì. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Nguyễn Đỗ Khánh Linh đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm. Điều cần lưu ý là các bài tự luận của em còn thiếu bước lập luận hoặc thiếu kết luận, dù hướng làm đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -566,7 +566,7 @@
         <v/>
       </c>
       <c r="E10" t="str">
-        <v>Trong Quý 1, em Nguyễn Hoàng Gia Linh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Kết quả của em tương đối đồng đều qua các lần kiểm tra, không có giai đoạn nào sa sút rõ rệt. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Nguyễn Hoàng Gia Linh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Nhiều câu em làm được một phần, cho thấy em đã nắm được hướng giải nhưng chưa hoàn thiện hết các ý. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -586,7 +586,7 @@
         <v/>
       </c>
       <c r="E11" t="str">
-        <v>Trong Quý 1, em Nguyễn Hoàng Minh Châu đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Kết quả của em tương đối đồng đều qua các lần kiểm tra, không có giai đoạn nào sa sút rõ rệt. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Nguyễn Hoàng Minh Châu đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Điều cần lưu ý là các bài tự luận của em còn thiếu bước lập luận hoặc thiếu kết luận, dù hướng làm đúng. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -606,7 +606,7 @@
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>Trong Quý 1, em Nguyễn Mai Anh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Kết quả giữa các lần kiểm tra của em có độ chênh khá lớn: có lần làm rất tốt nhưng cũng có lần còn ở mức thấp, cho thấy phong độ chưa thật ổn định. Em có kết quả khá nhất ở vectơ và các phép toán vectơ.</v>
+        <v>Trong Quý 1, em Nguyễn Mai Anh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Em thường làm đúng hướng nhưng dừng ở mức một phần các câu tự luận. Em có kết quả khá nhất ở vectơ và các phép toán vectơ.</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -626,7 +626,7 @@
         <v/>
       </c>
       <c r="E13" t="str">
-        <v>Trong Quý 1, em Nguyễn Ngọc Diễm đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Kết quả các bài cuối quý có phần giảm so với giai đoạn đầu, rất có thể do khối lượng kiến thức tăng nhanh ở giai đoạn ôn thi giữa kì. Em đạt kết quả cao nhất ở giá trị lượng giác của góc từ 0° đến 180°. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Nguyễn Ngọc Diễm đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Khi làm bài, em còn để trống một số câu, phần lớn rơi vào các câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở giá trị lượng giác của góc từ 0° đến 180°. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -646,7 +646,7 @@
         <v/>
       </c>
       <c r="E14" t="str">
-        <v>Trong Quý 1, em Nguyễn Nhật Huy đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Điểm nổi bật là em làm tốt hơn hẳn khi kiểm tra tập trung so với luyện tập thường ngày, cho thấy em có khả năng huy động kiến thức dưới áp lực thời gian. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Nguyễn Nhật Huy đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Em thường làm đúng hướng nhưng dừng ở mức một phần các câu tự luận. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -666,7 +666,7 @@
         <v/>
       </c>
       <c r="E15" t="str">
-        <v>Trong Quý 1, em Nguyễn Phước Nam Phong đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Kết quả các bài cuối quý có phần giảm so với giai đoạn đầu, rất có thể do khối lượng kiến thức tăng nhanh ở giai đoạn ôn thi giữa kì. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Nguyễn Phước Nam Phong đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Điều cần lưu ý là các bài tự luận của em còn thiếu bước lập luận hoặc thiếu kết luận, dù hướng làm đúng. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F15" t="str">
         <v/>
@@ -686,7 +686,7 @@
         <v/>
       </c>
       <c r="E16" t="str">
-        <v>Trong Quý 1, em Phạm Minh Châu đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Kết quả các bài cuối quý có phần giảm so với giai đoạn đầu, rất có thể do khối lượng kiến thức tăng nhanh ở giai đoạn ôn thi giữa kì. Em thực hiện tốt các dạng bài của giá trị lượng giác của góc từ 0° đến 180°.</v>
+        <v>Trong Quý 1, em Phạm Minh Châu đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Khi làm bài, em còn để trống một số câu, phần lớn rơi vào các câu khó hoặc câu cuối đề. Em thực hiện tốt các dạng bài của giá trị lượng giác của góc từ 0° đến 180°.</v>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -706,7 +706,7 @@
         <v/>
       </c>
       <c r="E17" t="str">
-        <v>Trong Quý 1, em Phạm Ngọc Linh Chi đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Điểm đáng ghi nhận là em có tiến bộ rõ rệt về sau: kết quả những bài cuối quý cao hơn hẳn giai đoạn đầu, cho thấy em đã điều chỉnh được cách học. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Phạm Ngọc Linh Chi đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Điều cần lưu ý là các bài tự luận của em còn thiếu bước lập luận hoặc thiếu kết luận, dù hướng làm đúng. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -726,7 +726,7 @@
         <v/>
       </c>
       <c r="E18" t="str">
-        <v>Trong Quý 1, em Trần Anh Thư đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Điểm đáng ghi nhận là em có tiến bộ rõ rệt về sau: kết quả những bài cuối quý cao hơn hẳn giai đoạn đầu, cho thấy em đã điều chỉnh được cách học. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Trần Anh Thư đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Nhiều câu em làm được một phần, cho thấy em đã nắm được hướng giải nhưng chưa hoàn thiện hết các ý. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -746,7 +746,7 @@
         <v/>
       </c>
       <c r="E19" t="str">
-        <v>Trong Quý 1, em Trần Hữu Bảo Nam đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Kết quả của em tương đối đồng đều qua các lần kiểm tra, không có giai đoạn nào sa sút rõ rệt. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Trần Hữu Bảo Nam đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Khi làm bài, em còn để trống một số câu, phần lớn rơi vào các câu khó hoặc câu cuối đề. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -766,7 +766,7 @@
         <v/>
       </c>
       <c r="E20" t="str">
-        <v>Trong Quý 1, em Trần Thùy Anh đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Kết quả các bài cuối quý có phần giảm so với giai đoạn đầu, rất có thể do khối lượng kiến thức tăng nhanh ở giai đoạn ôn thi giữa kì. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Trần Thùy Anh đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Khi làm bài, em còn để trống một số câu, phần lớn rơi vào các câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -786,7 +786,7 @@
         <v/>
       </c>
       <c r="E21" t="str">
-        <v>Trong Quý 1, em Trịnh Bảo Nam đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Kết quả của em tương đối đồng đều qua các lần kiểm tra, không có giai đoạn nào sa sút rõ rệt. Em thực hiện tốt các dạng bài của vectơ và các phép toán vectơ.</v>
+        <v>Trong Quý 1, em Trịnh Bảo Nam đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Nhiều câu em làm được một phần, cho thấy em đã nắm được hướng giải nhưng chưa hoàn thiện hết các ý. Em thực hiện tốt các dạng bài của vectơ và các phép toán vectơ.</v>
       </c>
       <c r="F21" t="str">
         <v/>
@@ -806,7 +806,7 @@
         <v/>
       </c>
       <c r="E22" t="str">
-        <v>Trong Quý 1, em Vũ Bảo An đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Kết quả các bài cuối quý có phần giảm so với giai đoạn đầu, rất có thể do khối lượng kiến thức tăng nhanh ở giai đoạn ôn thi giữa kì. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Vũ Bảo An đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em thường làm đúng hướng nhưng dừng ở mức một phần các câu tự luận. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F22" t="str">
         <v/>
@@ -826,7 +826,7 @@
         <v/>
       </c>
       <c r="E23" t="str">
-        <v>Trong Quý 1, em Vũ Nhật Anh đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Điểm nổi bật là em làm tốt hơn hẳn khi kiểm tra tập trung so với luyện tập thường ngày, cho thấy em có khả năng huy động kiến thức dưới áp lực thời gian. Em đạt kết quả cao nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Vũ Nhật Anh đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Khi làm bài, em còn để trống một số câu, phần lớn rơi vào các câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F23" t="str">
         <v/>

</xml_diff>

<commit_message>
feat(qa): nhan xet Q1 dung error-type cu the tung cau (khong dung nhom chung)
</commit_message>
<xml_diff>
--- a/docs/qa/10Olinda_Q1_nhan-xet.xlsx
+++ b/docs/qa/10Olinda_Q1_nhan-xet.xlsx
@@ -466,7 +466,7 @@
         <v/>
       </c>
       <c r="E5" t="str">
-        <v>Trong Quý 1, em Hoàng Anh Hà Chi đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Điều cần lưu ý là các bài tự luận của em còn thiếu bước lập luận hoặc thiếu kết luận, dù hướng làm đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Hoàng Anh Hà Chi đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F5" t="str">
         <v/>
@@ -486,7 +486,7 @@
         <v/>
       </c>
       <c r="E6" t="str">
-        <v>Trong Quý 1, em Hoàng Tuấn Minh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Khi làm bài, em còn để trống một số câu, phần lớn rơi vào các câu khó hoặc câu cuối đề. Em có kết quả khá nhất ở vectơ và các phép toán vectơ.</v>
+        <v>Trong Quý 1, em Hoàng Tuấn Minh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em có kết quả khá nhất ở vectơ và các phép toán vectơ.</v>
       </c>
       <c r="F6" t="str">
         <v/>
@@ -506,7 +506,7 @@
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>Trong Quý 1, em Hồ Khánh Phương đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Đáng chú ý là phần lớn câu hỏi em đều làm đúng, số câu sai không nhiều và thường chỉ là lỗi nhỏ. Em nắm vững và vận dụng tốt nhất vectơ và các phép toán vectơ, bài làm thể hiện sự chính xác và trình bày rõ ràng.</v>
+        <v>Trong Quý 1, em Hồ Khánh Phương đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em nắm vững và vận dụng tốt nhất vectơ và các phép toán vectơ, bài thi thể hiện sự chính xác và trình bày rõ ràng.</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -526,7 +526,7 @@
         <v/>
       </c>
       <c r="E8" t="str">
-        <v>Trong Quý 1, em Nguyễn Công Bảo Khánh đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Điều cần lưu ý là các bài tự luận của em còn thiếu bước lập luận hoặc thiếu kết luận, dù hướng làm đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Nguyễn Công Bảo Khánh đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -546,7 +546,7 @@
         <v/>
       </c>
       <c r="E9" t="str">
-        <v>Trong Quý 1, em Nguyễn Đỗ Khánh Linh đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm. Điều cần lưu ý là các bài tự luận của em còn thiếu bước lập luận hoặc thiếu kết luận, dù hướng làm đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Nguyễn Đỗ Khánh Linh đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -566,7 +566,7 @@
         <v/>
       </c>
       <c r="E10" t="str">
-        <v>Trong Quý 1, em Nguyễn Hoàng Gia Linh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Nhiều câu em làm được một phần, cho thấy em đã nắm được hướng giải nhưng chưa hoàn thiện hết các ý. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Nguyễn Hoàng Gia Linh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -586,7 +586,7 @@
         <v/>
       </c>
       <c r="E11" t="str">
-        <v>Trong Quý 1, em Nguyễn Hoàng Minh Châu đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Điều cần lưu ý là các bài tự luận của em còn thiếu bước lập luận hoặc thiếu kết luận, dù hướng làm đúng. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Nguyễn Hoàng Minh Châu đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -606,7 +606,7 @@
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>Trong Quý 1, em Nguyễn Mai Anh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Em thường làm đúng hướng nhưng dừng ở mức một phần các câu tự luận. Em có kết quả khá nhất ở vectơ và các phép toán vectơ.</v>
+        <v>Trong Quý 1, em Nguyễn Mai Anh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em có kết quả khá nhất ở vectơ và các phép toán vectơ.</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -626,7 +626,7 @@
         <v/>
       </c>
       <c r="E13" t="str">
-        <v>Trong Quý 1, em Nguyễn Ngọc Diễm đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Khi làm bài, em còn để trống một số câu, phần lớn rơi vào các câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở giá trị lượng giác của góc từ 0° đến 180°. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Nguyễn Ngọc Diễm đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở giá trị lượng giác của góc từ 0° đến 180°. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -646,7 +646,7 @@
         <v/>
       </c>
       <c r="E14" t="str">
-        <v>Trong Quý 1, em Nguyễn Nhật Huy đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Em thường làm đúng hướng nhưng dừng ở mức một phần các câu tự luận. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Nguyễn Nhật Huy đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -666,7 +666,7 @@
         <v/>
       </c>
       <c r="E15" t="str">
-        <v>Trong Quý 1, em Nguyễn Phước Nam Phong đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Điều cần lưu ý là các bài tự luận của em còn thiếu bước lập luận hoặc thiếu kết luận, dù hướng làm đúng. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Nguyễn Phước Nam Phong đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F15" t="str">
         <v/>
@@ -686,7 +686,7 @@
         <v/>
       </c>
       <c r="E16" t="str">
-        <v>Trong Quý 1, em Phạm Minh Châu đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Khi làm bài, em còn để trống một số câu, phần lớn rơi vào các câu khó hoặc câu cuối đề. Em thực hiện tốt các dạng bài của giá trị lượng giác của góc từ 0° đến 180°.</v>
+        <v>Trong Quý 1, em Phạm Minh Châu đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em thực hiện tốt các dạng bài của giá trị lượng giác của góc từ 0° đến 180°.</v>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -706,7 +706,7 @@
         <v/>
       </c>
       <c r="E17" t="str">
-        <v>Trong Quý 1, em Phạm Ngọc Linh Chi đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Điều cần lưu ý là các bài tự luận của em còn thiếu bước lập luận hoặc thiếu kết luận, dù hướng làm đúng. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Phạm Ngọc Linh Chi đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -726,7 +726,7 @@
         <v/>
       </c>
       <c r="E18" t="str">
-        <v>Trong Quý 1, em Trần Anh Thư đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Nhiều câu em làm được một phần, cho thấy em đã nắm được hướng giải nhưng chưa hoàn thiện hết các ý. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Trần Anh Thư đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -746,7 +746,7 @@
         <v/>
       </c>
       <c r="E19" t="str">
-        <v>Trong Quý 1, em Trần Hữu Bảo Nam đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Khi làm bài, em còn để trống một số câu, phần lớn rơi vào các câu khó hoặc câu cuối đề. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Trần Hữu Bảo Nam đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -766,7 +766,7 @@
         <v/>
       </c>
       <c r="E20" t="str">
-        <v>Trong Quý 1, em Trần Thùy Anh đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Khi làm bài, em còn để trống một số câu, phần lớn rơi vào các câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Trần Thùy Anh đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -786,7 +786,7 @@
         <v/>
       </c>
       <c r="E21" t="str">
-        <v>Trong Quý 1, em Trịnh Bảo Nam đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Nhiều câu em làm được một phần, cho thấy em đã nắm được hướng giải nhưng chưa hoàn thiện hết các ý. Em thực hiện tốt các dạng bài của vectơ và các phép toán vectơ.</v>
+        <v>Trong Quý 1, em Trịnh Bảo Nam đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em thực hiện tốt các dạng bài của vectơ và các phép toán vectơ.</v>
       </c>
       <c r="F21" t="str">
         <v/>
@@ -806,7 +806,7 @@
         <v/>
       </c>
       <c r="E22" t="str">
-        <v>Trong Quý 1, em Vũ Bảo An đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Em thường làm đúng hướng nhưng dừng ở mức một phần các câu tự luận. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Vũ Bảo An đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F22" t="str">
         <v/>
@@ -826,7 +826,7 @@
         <v/>
       </c>
       <c r="E23" t="str">
-        <v>Trong Quý 1, em Vũ Nhật Anh đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Khi làm bài, em còn để trống một số câu, phần lớn rơi vào các câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Vũ Nhật Anh đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F23" t="str">
         <v/>

</xml_diff>

<commit_message>
feat(qa): xep loai nhan xet theo diem thi giua HKI, doi trung binh thanh co ban
</commit_message>
<xml_diff>
--- a/docs/qa/10Olinda_Q1_nhan-xet.xlsx
+++ b/docs/qa/10Olinda_Q1_nhan-xet.xlsx
@@ -466,7 +466,7 @@
         <v/>
       </c>
       <c r="E5" t="str">
-        <v>Trong Quý 1, em Hoàng Anh Hà Chi đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Hoàng Anh Hà Chi đạt kết quả học tập môn Toán ở mức khá tốt, nắm chắc các nội dung trọng tâm của chương trình. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F5" t="str">
         <v/>
@@ -486,7 +486,7 @@
         <v/>
       </c>
       <c r="E6" t="str">
-        <v>Trong Quý 1, em Hoàng Tuấn Minh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em có kết quả khá nhất ở vectơ và các phép toán vectơ.</v>
+        <v>Trong Quý 1, em Hoàng Tuấn Minh đạt kết quả học tập môn Toán ở mức cơ bản, đã tiếp cận được các kiến thức nền của chương trình. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em có kết quả khá nhất ở vectơ và các phép toán vectơ.</v>
       </c>
       <c r="F6" t="str">
         <v/>
@@ -506,7 +506,7 @@
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>Trong Quý 1, em Hồ Khánh Phương đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em nắm vững và vận dụng tốt nhất vectơ và các phép toán vectơ, bài thi thể hiện sự chính xác và trình bày rõ ràng.</v>
+        <v>Trong Quý 1, em Hồ Khánh Phương đạt kết quả học tập môn Toán ở mức khá tốt, nắm chắc các nội dung trọng tâm của chương trình. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em nắm vững và vận dụng tốt nhất vectơ và các phép toán vectơ, bài thi thể hiện sự chính xác và trình bày rõ ràng.</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -526,7 +526,7 @@
         <v/>
       </c>
       <c r="E8" t="str">
-        <v>Trong Quý 1, em Nguyễn Công Bảo Khánh đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Nguyễn Công Bảo Khánh đạt kết quả học tập môn Toán ở mức tốt, bài kiểm tra giữa học kì cho thấy nền tảng kiến thức vững và khả năng vận dụng thành thạo. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -546,7 +546,7 @@
         <v/>
       </c>
       <c r="E9" t="str">
-        <v>Trong Quý 1, em Nguyễn Đỗ Khánh Linh đạt kết quả học tập môn Toán ở mức khá, nắm được phần lớn kiến thức trọng tâm. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Nguyễn Đỗ Khánh Linh đạt kết quả học tập môn Toán ở mức khá, đã nắm được phần lớn kiến thức của chương trình. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -566,7 +566,7 @@
         <v/>
       </c>
       <c r="E10" t="str">
-        <v>Trong Quý 1, em Nguyễn Hoàng Gia Linh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Nguyễn Hoàng Gia Linh đạt kết quả học tập môn Toán ở mức khá, đã nắm được phần lớn kiến thức của chương trình. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -586,7 +586,7 @@
         <v/>
       </c>
       <c r="E11" t="str">
-        <v>Trong Quý 1, em Nguyễn Hoàng Minh Châu đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Nguyễn Hoàng Minh Châu đạt kết quả học tập môn Toán ở mức cơ bản, đã tiếp cận được các kiến thức nền của chương trình. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em có kết quả khá nhất ở mệnh đề và các phép suy luận toán học. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -606,7 +606,7 @@
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>Trong Quý 1, em Nguyễn Mai Anh đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em có kết quả khá nhất ở vectơ và các phép toán vectơ.</v>
+        <v>Trong Quý 1, em Nguyễn Mai Anh đạt kết quả học tập môn Toán ở mức cơ bản, đã tiếp cận được các kiến thức nền của chương trình. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em có kết quả khá nhất ở vectơ và các phép toán vectơ.</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -626,7 +626,7 @@
         <v/>
       </c>
       <c r="E13" t="str">
-        <v>Trong Quý 1, em Nguyễn Ngọc Diễm đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở giá trị lượng giác của góc từ 0° đến 180°. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Nguyễn Ngọc Diễm bước đầu làm quen với các nội dung của chương trình Toán và đã tham gia đầy đủ các giờ học. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở giá trị lượng giác của góc từ 0° đến 180°. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -646,7 +646,7 @@
         <v/>
       </c>
       <c r="E14" t="str">
-        <v>Trong Quý 1, em Nguyễn Nhật Huy đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Nguyễn Nhật Huy đạt kết quả học tập môn Toán ở mức khá tốt, nắm chắc các nội dung trọng tâm của chương trình. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -666,7 +666,7 @@
         <v/>
       </c>
       <c r="E15" t="str">
-        <v>Trong Quý 1, em Nguyễn Phước Nam Phong đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Nguyễn Phước Nam Phong đạt kết quả học tập môn Toán ở mức khá, đã nắm được phần lớn kiến thức của chương trình. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F15" t="str">
         <v/>
@@ -686,7 +686,7 @@
         <v/>
       </c>
       <c r="E16" t="str">
-        <v>Trong Quý 1, em Phạm Minh Châu đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em thực hiện tốt các dạng bài của giá trị lượng giác của góc từ 0° đến 180°.</v>
+        <v>Trong Quý 1, em Phạm Minh Châu đạt kết quả học tập môn Toán ở mức cơ bản, đã tiếp cận được các kiến thức nền của chương trình. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em thực hiện tốt các dạng bài của giá trị lượng giác của góc từ 0° đến 180°.</v>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -706,7 +706,7 @@
         <v/>
       </c>
       <c r="E17" t="str">
-        <v>Trong Quý 1, em Phạm Ngọc Linh Chi đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Phạm Ngọc Linh Chi đạt kết quả học tập môn Toán ở mức khá, đã nắm được phần lớn kiến thức của chương trình. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -726,7 +726,7 @@
         <v/>
       </c>
       <c r="E18" t="str">
-        <v>Trong Quý 1, em Trần Anh Thư đạt kết quả học tập môn Toán ở mức khá, giữ được nhịp học đều đặn. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
+        <v>Trong Quý 1, em Trần Anh Thư đạt kết quả học tập môn Toán ở mức khá, đã nắm được phần lớn kiến thức của chương trình. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em thực hiện tốt các dạng bài của mệnh đề và các phép suy luận toán học.</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -746,7 +746,7 @@
         <v/>
       </c>
       <c r="E19" t="str">
-        <v>Trong Quý 1, em Trần Hữu Bảo Nam đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Trần Hữu Bảo Nam đạt kết quả học tập môn Toán ở mức cơ bản, đã tiếp cận được các kiến thức nền của chương trình. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em có kết quả khá nhất ở vectơ và các phép toán vectơ. Nội dung bất phương trình và hệ bất phương trình bậc nhất hai ẩn cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -766,7 +766,7 @@
         <v/>
       </c>
       <c r="E20" t="str">
-        <v>Trong Quý 1, em Trần Thùy Anh đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Trần Thùy Anh đạt kết quả học tập môn Toán ở mức cơ bản, đã tiếp cận được các kiến thức nền của chương trình. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -786,7 +786,7 @@
         <v/>
       </c>
       <c r="E21" t="str">
-        <v>Trong Quý 1, em Trịnh Bảo Nam đạt kết quả học tập môn Toán ở mức trung bình, đã nắm được các kiến thức cơ bản của chương trình. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em thực hiện tốt các dạng bài của vectơ và các phép toán vectơ.</v>
+        <v>Trong Quý 1, em Trịnh Bảo Nam đạt kết quả học tập môn Toán ở mức khá, đã nắm được phần lớn kiến thức của chương trình. Trong quá trình đánh giá, ở các câu tự luận còn thiếu bước lập luận hoặc chưa có kết luận, dù hướng giải đúng. Em thực hiện tốt các dạng bài của vectơ và các phép toán vectơ.</v>
       </c>
       <c r="F21" t="str">
         <v/>
@@ -806,7 +806,7 @@
         <v/>
       </c>
       <c r="E22" t="str">
-        <v>Trong Quý 1, em Vũ Bảo An đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Vũ Bảo An bước đầu làm quen với các nội dung của chương trình Toán và đã tham gia đầy đủ các giờ học. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở mệnh đề và các phép suy luận toán học. Nội dung vectơ và các phép toán vectơ cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F22" t="str">
         <v/>
@@ -826,7 +826,7 @@
         <v/>
       </c>
       <c r="E23" t="str">
-        <v>Trong Quý 1, em Vũ Nhật Anh đã tham gia học tập và bước đầu làm quen với các nội dung của chương trình Toán. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
+        <v>Trong Quý 1, em Vũ Nhật Anh đạt kết quả học tập môn Toán ở mức cơ bản, đã tiếp cận được các kiến thức nền của chương trình. Trong quá trình đánh giá, còn để trống một số câu, phần lớn rơi vào những câu khó hoặc câu cuối đề. Em đạt kết quả cao nhất ở vectơ và các phép toán vectơ. Nội dung hệ thức lượng trong tam giác cần được củng cố và rèn luyện thêm.</v>
       </c>
       <c r="F23" t="str">
         <v/>

</xml_diff>